<commit_message>
PO upload handling with shelf life
</commit_message>
<xml_diff>
--- a/assets/csv/sample_purchase_order.xlsx
+++ b/assets/csv/sample_purchase_order.xlsx
@@ -1,16 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
-  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aleemktk/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\avenzur\assets\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71F033D8-CD13-2941-ABCF-A031C7337E22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="23260" windowHeight="12460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="23260" windowHeight="12460"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,12 +16,12 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$T$2</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>Item Bar code.</t>
   </si>
@@ -49,6 +47,15 @@
     <t>Qty</t>
   </si>
   <si>
+    <t>Sale Price (without VAT)</t>
+  </si>
+  <si>
+    <t>Purchase Price (without VAT)</t>
+  </si>
+  <si>
+    <t>Cost Price (without VAT)</t>
+  </si>
+  <si>
     <t>Vat %</t>
   </si>
   <si>
@@ -74,6 +81,9 @@
   </si>
   <si>
     <t xml:space="preserve">Image link </t>
+  </si>
+  <si>
+    <t>Shelf Life</t>
   </si>
   <si>
     <r>
@@ -81,10 +91,11 @@
     </r>
     <r>
       <rPr>
-        <b/>
+        <rFont val="Aptos Narrow"/>
+        <b val="1"/>
+        <color theme="1"/>
         <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
+        <scheme val="none"/>
       </rPr>
       <t xml:space="preserve">
 باور عالي التركيز توتال وور 30 حصة</t>
@@ -106,25 +117,19 @@
     <t>https://proteinpackage.co.uk/cdn/shop/files/Total-War-Pump-Blue-Lemonade-Pre-Workout-310g_1000x.png?v=1723204123</t>
   </si>
   <si>
-    <t>Cost Price (without VAT)</t>
-  </si>
-  <si>
-    <t>Purchase Price (without VAT)</t>
-  </si>
-  <si>
-    <t>Sale Price (without VAT)</t>
+    <t>one week</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="[$-409]mmm\-yy;@"/>
-    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="[$-409]mmm-yy;@"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* (#,##0.00);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* (#,##0.00);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,7 +147,6 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -155,13 +159,6 @@
       <sz val="11"/>
       <color theme="10"/>
       <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -180,7 +177,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <fgColor theme="2" tint="-0.0999786370433668"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -204,13 +201,7 @@
     </fill>
   </fills>
   <borders count="2">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
     <border>
       <left style="thin">
         <color indexed="64"/>
@@ -224,14 +215,13 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="17">
@@ -286,11 +276,11 @@
     </xf>
   </cellXfs>
   <cellStyles count="5">
-    <cellStyle name="Comma 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
+    <cellStyle name="Comma 2" xfId="2"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Hyperlink" xfId="4" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -302,14 +292,6 @@
       <color rgb="FFCC99FF"/>
     </mruColors>
   </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -318,10 +300,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -601,38 +583,36 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="21.1640625" customWidth="1"/>
+    <col min="1" max="1" width="21.19922" customWidth="1"/>
     <col min="2" max="2" width="72" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="5" width="16.1640625" customWidth="1"/>
-    <col min="6" max="6" width="12.1640625" customWidth="1"/>
+    <col min="3" max="3" width="18.79688" customWidth="1"/>
+    <col min="4" max="5" width="16.19922" customWidth="1"/>
+    <col min="6" max="6" width="12.19922" customWidth="1"/>
     <col min="7" max="7" width="15.5" customWidth="1"/>
-    <col min="8" max="8" width="9.83203125" customWidth="1"/>
+    <col min="8" max="8" width="9.796875" customWidth="1"/>
     <col min="9" max="9" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.69922" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
-    <col min="12" max="12" width="7.83203125" customWidth="1"/>
-    <col min="13" max="13" width="7.1640625" customWidth="1"/>
-    <col min="14" max="14" width="8.1640625" customWidth="1"/>
+    <col min="12" max="12" width="7.796875" customWidth="1"/>
+    <col min="13" max="13" width="7.199219" customWidth="1"/>
+    <col min="14" max="14" width="8.199219" customWidth="1"/>
     <col min="15" max="15" width="8.5" customWidth="1"/>
     <col min="16" max="16" width="7.5" customWidth="1"/>
     <col min="17" max="17" width="8.5" customWidth="1"/>
-    <col min="18" max="18" width="5.83203125" customWidth="1"/>
-    <col min="19" max="19" width="114.1640625" customWidth="1"/>
-    <col min="20" max="20" width="103.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="5.796875" customWidth="1"/>
+    <col min="19" max="19" width="114.1992" customWidth="1"/>
+    <col min="20" max="20" width="103.2969" style="3" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.89844" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="1" customFormat="1" ht="37.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" s="1" customFormat="1" ht="37.25" customHeight="1">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -658,52 +638,55 @@
         <v>7</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>16</v>
+        <v>19</v>
+      </c>
+      <c r="U1" s="4" t="s">
+        <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:20" s="2" customFormat="1" ht="49.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" s="2" customFormat="1" ht="49.25" customHeight="1">
       <c r="A2" s="6">
         <v>850004759189</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C2" s="8"/>
       <c r="D2" s="8" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E2" s="9"/>
       <c r="F2" s="8"/>
@@ -728,17 +711,19 @@
       <c r="Q2" s="11"/>
       <c r="R2" s="11"/>
       <c r="S2" s="15" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="T2" s="16" t="s">
-        <v>20</v>
+        <v>24</v>
+      </c>
+      <c r="U2" s="11" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="T2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="T2" r:id="rId1"/>
   </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup r:id="rId2" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
PO upload fixed wiyh new xlxs requiremnets
</commit_message>
<xml_diff>
--- a/assets/csv/sample_purchase_order.xlsx
+++ b/assets/csv/sample_purchase_order.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\avenzur\assets\csv\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="23260" windowHeight="12460"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -103,6 +103,9 @@
   </si>
   <si>
     <t>BLUE LEMONADE</t>
+  </si>
+  <si>
+    <t>aaaa</t>
   </si>
   <si>
     <t>Total War is pre-workout designed with high-quality ingredients packed with caffeine, green tea, beta-alanine, and juniper berries that provide you with unstoppable strength to help you take control of even the toughest workouts.
@@ -168,12 +171,18 @@
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -224,7 +233,7 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -238,40 +247,46 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="4" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="2" fillId="5" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -588,50 +603,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="21.19922" customWidth="1"/>
     <col min="2" max="2" width="72" customWidth="1"/>
     <col min="3" max="3" width="18.79688" customWidth="1"/>
     <col min="4" max="5" width="16.19922" customWidth="1"/>
     <col min="6" max="6" width="12.19922" customWidth="1"/>
-    <col min="7" max="7" width="15.5" customWidth="1"/>
+    <col min="7" max="7" width="15.39844" customWidth="1"/>
     <col min="8" max="8" width="9.796875" customWidth="1"/>
-    <col min="9" max="9" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.39844" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.69922" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
     <col min="12" max="12" width="7.796875" customWidth="1"/>
     <col min="13" max="13" width="7.199219" customWidth="1"/>
     <col min="14" max="14" width="8.199219" customWidth="1"/>
-    <col min="15" max="15" width="8.5" customWidth="1"/>
-    <col min="16" max="16" width="7.5" customWidth="1"/>
-    <col min="17" max="17" width="8.5" customWidth="1"/>
+    <col min="15" max="15" width="8.398438" customWidth="1"/>
+    <col min="16" max="16" width="7.398438" customWidth="1"/>
+    <col min="17" max="17" width="8.398438" customWidth="1"/>
     <col min="18" max="18" width="5.796875" customWidth="1"/>
     <col min="19" max="19" width="114.1992" customWidth="1"/>
     <col min="20" max="20" width="103.2969" style="3" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="16.89844" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="37.25" customHeight="1">
+    <row r="1" s="1" customFormat="1" ht="37.2" customHeight="1">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="4" t="s">
@@ -649,22 +664,22 @@
       <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="Q1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="R1" s="5" t="s">
         <v>17</v>
       </c>
       <c r="S1" s="4" t="s">
@@ -673,51 +688,57 @@
       <c r="T1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="U1" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" s="2" customFormat="1" ht="49.25" customHeight="1">
-      <c r="A2" s="6">
+    <row r="2" s="2" customFormat="1" ht="49.2" customHeight="1">
+      <c r="A2" s="8">
         <v>850004759189</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8" t="s">
+      <c r="C2" s="10"/>
+      <c r="D2" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="E2" s="9"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="10">
+      <c r="E2" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="10"/>
+      <c r="G2" s="12">
         <v>46722</v>
       </c>
-      <c r="H2" s="11">
+      <c r="H2" s="13">
         <v>12</v>
       </c>
-      <c r="I2" s="12">
+      <c r="I2" s="14">
         <v>138</v>
       </c>
-      <c r="J2" s="9"/>
-      <c r="K2" s="13">
+      <c r="J2" s="11">
+        <v>1111</v>
+      </c>
+      <c r="K2" s="15">
         <v>75</v>
       </c>
-      <c r="L2" s="9"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="11"/>
-      <c r="O2" s="11"/>
-      <c r="P2" s="11"/>
-      <c r="Q2" s="11"/>
-      <c r="R2" s="11"/>
-      <c r="S2" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="T2" s="16" t="s">
+      <c r="L2" s="11">
+        <v>15</v>
+      </c>
+      <c r="M2" s="16"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="U2" s="11" t="s">
+      <c r="T2" s="18" t="s">
         <v>25</v>
+      </c>
+      <c r="U2" s="13" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>